<commit_message>
Added PTAR_ACH test case
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/Reporting.xlsx
+++ b/KatalonData/Bootstrap/Reporting.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="89">
   <si>
     <t>Result</t>
   </si>
@@ -278,6 +278,24 @@
   </si>
   <si>
     <t>Wed Sep 16 22:36:02 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 19:28:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 20:12:31 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 20:28:37 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 20:42:05 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 21:04:45 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Sep 17 21:24:50 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1028,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="3" t="s">
@@ -1104,7 +1122,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>12</v>

</xml_diff>

<commit_message>
Online Reporting Test Cases
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/Reporting.xlsx
+++ b/KatalonData/Bootstrap/Reporting.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDDE5BC-FE62-4F68-9529-49F683021837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8F6611-6FFB-488A-9657-108F39D7F7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1776" yWindow="1776" windowWidth="17280" windowHeight="9972" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9972" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="APPR" sheetId="1" r:id="rId1"/>
@@ -21,11 +21,13 @@
     <sheet name="PR_SR_ACH_Fail" sheetId="11" r:id="rId6"/>
     <sheet name="PR_SR_PC" sheetId="5" r:id="rId7"/>
     <sheet name="PR_SR_Corp" sheetId="12" r:id="rId8"/>
-    <sheet name="PR_SR_PS" sheetId="13" r:id="rId9"/>
-    <sheet name="SPR_Deferred_CC" sheetId="6" r:id="rId10"/>
-    <sheet name="SPR_Autopay_CC" sheetId="7" r:id="rId11"/>
-    <sheet name="SPR_Deferred_PC" sheetId="8" r:id="rId12"/>
-    <sheet name="SPR_Autopay_ACH" sheetId="9" r:id="rId13"/>
+    <sheet name="PR_SR_Corp_Fail" sheetId="14" r:id="rId9"/>
+    <sheet name="PR_SR_PS" sheetId="13" r:id="rId10"/>
+    <sheet name="PR_SR_PS_Fail" sheetId="15" r:id="rId11"/>
+    <sheet name="SPR_Deferred_CC" sheetId="6" r:id="rId12"/>
+    <sheet name="SPR_Autopay_CC" sheetId="7" r:id="rId13"/>
+    <sheet name="SPR_Deferred_PC" sheetId="8" r:id="rId14"/>
+    <sheet name="SPR_Autopay_ACH" sheetId="9" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="95">
   <si>
     <t>Result</t>
   </si>
@@ -279,55 +281,49 @@
     <t>Fri Oct 09 20:48:28 IST 2026</t>
   </si>
   <si>
-    <t>Mon Oct 12 21:11:53 IST 2026</t>
-  </si>
-  <si>
     <t>10.11</t>
   </si>
   <si>
     <t>Thu Oct 15 20:14:35 IST 2026</t>
   </si>
   <si>
-    <t>Wed Oct 21 00:46:38 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Oct 21 16:23:39 IST 2026</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Wed Oct 21 21:23:58 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Oct 21 21:26:52 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Oct 21 21:57:17 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Oct 21 22:40:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Wed Oct 21 22:48:29 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Oct 22 21:02:44 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Oct 22 21:25:32 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Oct 22 21:38:54 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Oct 22 21:54:53 IST 2026</t>
-  </si>
-  <si>
-    <t>Thu Oct 22 22:21:36 IST 2026</t>
-  </si>
-  <si>
     <t>Thu Oct 22 22:25:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Fri Oct 23 22:08:57 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Oct 26 19:24:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Oct 26 20:03:25 IST 2026</t>
+  </si>
+  <si>
+    <t>10.02</t>
+  </si>
+  <si>
+    <t>Mon Oct 26 22:05:04 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 19:19:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 19:33:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:41:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Oct 27 21:45:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 28 21:17:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 28 21:34:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Wed Oct 28 21:44:17 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -792,6 +788,194 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AB6CEF-06F8-4D48-B1DE-C9E09F6E39EC}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FAE3C7F-63D6-4130-9E47-C1659FC62247}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45CC1875-7BF0-42BA-B234-4151711F71DE}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -890,7 +1074,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFBB72D0-0860-41BA-B858-39B81B6416AB}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -984,7 +1168,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20515725-403B-4344-8B9C-3754B0847C97}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1083,7 +1267,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A68AE674-98FB-40CB-A6EE-AC4C15F830D5}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1456,7 +1640,7 @@
         <v>73</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="3" t="s">
@@ -1472,7 +1656,7 @@
         <v>65</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>33</v>
@@ -1642,7 +1826,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>12</v>
@@ -1731,10 +1915,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s" s="0">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="3" t="s">
@@ -1775,7 +1959,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AB6CEF-06F8-4D48-B1DE-C9E09F6E39EC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA28B56-4796-426B-AEAE-FE1834C0D198}">
   <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1825,10 +2009,10 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s" s="0">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="3" t="s">
@@ -1844,20 +2028,20 @@
         <v>65</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="I2" s="3" t="s">
         <v>33</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>37</v>

</xml_diff>